<commit_message>
modifique el modelo xlsxdrive y agregue un el archivo drive_manager.py
</commit_message>
<xml_diff>
--- a/LISTAS/ma/FILTRO PARA SPAR DISMAY.xlsx
+++ b/LISTAS/ma/FILTRO PARA SPAR DISMAY.xlsx
@@ -761,14 +761,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="15" t="n">
-        <v>45194.64992091935</v>
+        <v>45217</v>
       </c>
       <c r="E1" s="4" t="n"/>
     </row>
-    <row r="2"/>
-    <row r="3"/>
-    <row r="4"/>
-    <row r="5"/>
     <row r="6" ht="22.5" customHeight="1" s="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
@@ -814,26 +810,6 @@
       </c>
       <c r="E11" s="7" t="n"/>
     </row>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
     <row r="32" ht="18" customHeight="1" s="1">
       <c r="A32" s="12" t="inlineStr">
         <is>
@@ -865,14 +841,11 @@
       </c>
       <c r="C33" s="23" t="n"/>
       <c r="D33" s="25" t="n">
-        <v>230</v>
+        <v>250</v>
       </c>
     </row>
     <row r="34" ht="16.5" customHeight="1" s="1"/>
     <row r="35" ht="16.5" customHeight="1" s="1"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
     <row r="39" ht="19.5" customHeight="1" s="1">
       <c r="A39" s="14" t="inlineStr">
         <is>
@@ -880,15 +853,12 @@
         </is>
       </c>
     </row>
-    <row r="40"/>
     <row r="41">
       <c r="A41" s="10" t="n"/>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" s="11" t="n"/>
     </row>
-    <row r="44"/>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
@@ -898,12 +868,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="A11:D11"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A9:D9"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A11:D11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>